<commit_message>
chore(dev-tools): add HTTP request samples, update gitignore and seed data
- Add .http file samples for testing catalog endpoints flow
- Update .gitignore rules for local dev environment
- Fix minor attribute inconsistencies in Excel seed data
- Adjust import directive order in user controller
</commit_message>
<xml_diff>
--- a/backend/Ecommerce/src/Modules/Products/Infrastructure/Data/SeedData.xlsx
+++ b/backend/Ecommerce/src/Modules/Products/Infrastructure/Data/SeedData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas Callamullo\Documents\Visual Studio Code\cs_ecommerce\backend\Ecommerce\src\Modules\Products\Infrastructure\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067CEF2D-E9DE-475E-9B85-DC9E776F006F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3146E8-D721-4A4D-B8BC-22EE012BA5E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1325,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>19</v>
@@ -1364,7 +1364,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="L14" s="1" t="s">
         <v>19</v>

</xml_diff>